<commit_message>
Lijst volgens nieuwe opvatting
#72
</commit_message>
<xml_diff>
--- a/prius2/input/ad-hoc_v25-08-19.xlsx
+++ b/prius2/input/ad-hoc_v25-08-19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bram_dhondt\Documents\GitHub\prius\prius2\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C03398F-4A6E-4697-900C-7748188B3B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197BC480-6D30-49A4-8510-5DDAAE83378D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>groep</t>
   </si>
@@ -40,12 +40,6 @@
     <t>plant</t>
   </si>
   <si>
-    <t>late guldenroede</t>
-  </si>
-  <si>
-    <t>Canadese guldenroede</t>
-  </si>
-  <si>
     <t>Gebaseerd op</t>
   </si>
   <si>
@@ -70,64 +64,46 @@
     <t>Amerikaanse rode eekhoorn</t>
   </si>
   <si>
+    <t>Vallisneria australis</t>
+  </si>
+  <si>
+    <t>halsbandparkiet</t>
+  </si>
+  <si>
+    <t>grote Alexanderparkiet</t>
+  </si>
+  <si>
+    <t>monniksparkiet</t>
+  </si>
+  <si>
+    <t>Turkse rivierkreeft</t>
+  </si>
+  <si>
+    <t>prachtslang</t>
+  </si>
+  <si>
+    <t>Aziatische tijgermug</t>
+  </si>
+  <si>
+    <t>Canadese gans</t>
+  </si>
+  <si>
+    <t>damhert</t>
+  </si>
+  <si>
+    <t>Procambarus zonangulus</t>
+  </si>
+  <si>
+    <t>Amynthas agrestis</t>
+  </si>
+  <si>
+    <t>Amynthas tokioensis</t>
+  </si>
+  <si>
+    <t>Metaphire hilgendorfi</t>
+  </si>
+  <si>
     <t>Hydrocharis laevigata</t>
-  </si>
-  <si>
-    <t>Lycium ferocissimum</t>
-  </si>
-  <si>
-    <t>gestreepte Amerikaanse rivierkreeft</t>
-  </si>
-  <si>
-    <t>Vallisneria australis</t>
-  </si>
-  <si>
-    <t>halsbandparkiet</t>
-  </si>
-  <si>
-    <t>grote Alexanderparkiet</t>
-  </si>
-  <si>
-    <t>monniksparkiet</t>
-  </si>
-  <si>
-    <t>Amerikaanse hondsvis</t>
-  </si>
-  <si>
-    <t>Turkse rivierkreeft</t>
-  </si>
-  <si>
-    <t>prachtslang</t>
-  </si>
-  <si>
-    <t>zwartbekgrondel</t>
-  </si>
-  <si>
-    <t>Kesslers grondel</t>
-  </si>
-  <si>
-    <t>marmergrondel</t>
-  </si>
-  <si>
-    <t>Pontische stroomgrondel</t>
-  </si>
-  <si>
-    <t>naakthalsgrondel</t>
-  </si>
-  <si>
-    <t>Kaukasische dwerggrondel</t>
-  </si>
-  <si>
-    <t>shimofurigrondel</t>
-  </si>
-  <si>
-    <t>naakte grondel</t>
-  </si>
-  <si>
-    <t>Aziatische tijgermug</t>
-  </si>
-  <si>
-    <t>Canadese gans</t>
   </si>
 </sst>
 </file>
@@ -173,8 +149,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -455,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="32.109375" bestFit="1" customWidth="1"/>
@@ -464,22 +440,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -488,68 +464,68 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>8790531</v>
+        <v>2437282</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>5220435</v>
+        <v>1651430</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>5389017</v>
+        <v>5232437</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>5389029</v>
+        <v>5220435</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>2437282</v>
+        <v>8790531</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -558,40 +534,40 @@
         <v>1</v>
       </c>
       <c r="D7">
-        <v>11055820</v>
+        <v>5229055</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>3797394</v>
+        <v>2479226</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>2227289</v>
+        <v>2479407</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
@@ -600,40 +576,40 @@
         <v>1</v>
       </c>
       <c r="D10">
-        <v>2865524</v>
+        <v>8889878</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11">
-        <v>2479226</v>
+        <v>8946295</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>5229055</v>
+        <v>2865524</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
         <v>20</v>
@@ -642,12 +618,12 @@
         <v>1</v>
       </c>
       <c r="D13">
-        <v>2479407</v>
+        <v>5220136</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
         <v>21</v>
@@ -656,12 +632,12 @@
         <v>1</v>
       </c>
       <c r="D14">
-        <v>5203111</v>
+        <v>2227231</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B15" t="s">
         <v>22</v>
@@ -670,12 +646,12 @@
         <v>1</v>
       </c>
       <c r="D15">
-        <v>8946295</v>
+        <v>9225458</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B16" t="s">
         <v>23</v>
@@ -684,12 +660,12 @@
         <v>1</v>
       </c>
       <c r="D16">
-        <v>8889878</v>
+        <v>9448251</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
@@ -698,12 +674,12 @@
         <v>1</v>
       </c>
       <c r="D17">
-        <v>2379089</v>
+        <v>8458912</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
@@ -712,122 +688,13 @@
         <v>1</v>
       </c>
       <c r="D18">
-        <v>4285968</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19">
-        <v>2379245</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>2379105</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21">
-        <v>5788062</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22">
-        <v>2375688</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23">
-        <v>2376461</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <v>5208832</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25">
-        <v>1651430</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
-      <c r="D26">
-        <v>5232437</v>
+        <v>11055820</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D23">
+    <sortCondition ref="B2:B23"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -843,21 +710,21 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45883</v>
       </c>
     </row>

</xml_diff>